<commit_message>
fix: remove colume history
</commit_message>
<xml_diff>
--- a/backend/exports/monthly_report_2026-01-01_2026-12-31.xlsx
+++ b/backend/exports/monthly_report_2026-01-01_2026-12-31.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="63" uniqueCount="34">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="65" uniqueCount="35">
   <si>
     <t>Member</t>
   </si>
@@ -111,6 +111,9 @@
   </si>
   <si>
     <t>Trương Việt Hưng</t>
+  </si>
+  <si>
+    <t>ádasdasd</t>
   </si>
   <si>
     <t>Rank</t>
@@ -494,7 +497,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E30"/>
+  <dimension ref="A1:E31"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="24" customWidth="1"/>
@@ -534,10 +537,10 @@
         <v>7</v>
       </c>
       <c r="B5">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="C5">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D5">
         <v>0</v>
@@ -551,10 +554,10 @@
         <v>8</v>
       </c>
       <c r="B6">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="C6">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D6">
         <v>0</v>
@@ -968,6 +971,23 @@
         <v>0</v>
       </c>
       <c r="E30">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="31" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
+        <v>33</v>
+      </c>
+      <c r="B31">
+        <v>0</v>
+      </c>
+      <c r="C31">
+        <v>0</v>
+      </c>
+      <c r="D31">
+        <v>0</v>
+      </c>
+      <c r="E31">
         <v>0</v>
       </c>
     </row>
@@ -979,7 +999,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:D27"/>
+  <dimension ref="A1:D28"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="24" customWidth="1"/>
@@ -997,12 +1017,12 @@
         <v>3</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B2">
         <v>2</v>
@@ -1016,7 +1036,7 @@
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B3">
         <v>0</v>
@@ -1362,6 +1382,20 @@
       </c>
       <c r="D27">
         <v>26</v>
+      </c>
+    </row>
+    <row r="28" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
+        <v>33</v>
+      </c>
+      <c r="B28">
+        <v>0</v>
+      </c>
+      <c r="C28">
+        <v>0</v>
+      </c>
+      <c r="D28">
+        <v>27</v>
       </c>
     </row>
   </sheetData>

</xml_diff>